<commit_message>
fix(M048 v3.2 handoff): sync MD section 3.6 + xlsx Table 8 with corrected drop-VI sens arm
Earlier patch updated the sensitivity_arms.csv and the README/DOCX but the
markdown findings doc and xlsx Table 8 still showed the buggy drop-Bethesda-VI
arm matching n=3,121 (identical to D arm). User flagged the mismatch.

This patch:
- Rebuilds MD section 3.6 sensitivity-arms table from the patched CSV with
  arms in canonical order (A,B,C,D,E,F,G); E now reads n=2,599, Black OR
  0.417 (0.341-0.509, p<0.0001), Asian OR 1.27 (0.85-1.90, p=0.24).
- Adds an explicit drop-VI bullet to the commentary calling out the prior
  string-matching bug.
- Reorders xlsx Table 8 rows so E sits between D and F instead of being
  appended to the end of the sheet.
- Re-zips the handoff package.
</commit_message>
<xml_diff>
--- a/M048_submission_package/m048_v32_handoff_package/03_tables_for_manuscript.xlsx
+++ b/M048_submission_package/m048_v32_handoff_package/03_tables_for_manuscript.xlsx
@@ -9080,9 +9080,6 @@
       <c r="D6" t="n">
         <v>0.6892</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9101,9 +9098,6 @@
       <c r="D7" t="n">
         <v>0.4528</v>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9166,11 +9160,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S048v3_F_TR4_only</t>
+          <t>S048v3_E_no_Bethesda_VI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>455</v>
+        <v>2599</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -9178,28 +9172,28 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.6273</v>
+        <v>0.4169</v>
       </c>
       <c r="E10" t="n">
-        <v>0.386</v>
+        <v>0.3415</v>
       </c>
       <c r="F10" t="n">
-        <v>1.0195</v>
+        <v>0.509</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.0598</t>
+          <t>0.0000</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S048v3_F_TR4_only</t>
+          <t>S048v3_E_no_Bethesda_VI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>455</v>
+        <v>2599</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -9207,28 +9201,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4.0744</v>
+        <v>1.2705</v>
       </c>
       <c r="E11" t="n">
-        <v>1.4673</v>
+        <v>0.8493000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>11.3139</v>
+        <v>1.9006</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.0070</t>
+          <t>0.2440</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S048v3_G_had_fna</t>
+          <t>S048v3_F_TR4_only</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2258</v>
+        <v>455</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -9236,28 +9230,28 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.5859</v>
+        <v>0.6273</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4671</v>
+        <v>0.386</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7351</v>
+        <v>1.0195</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0598</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S048v3_G_had_fna</t>
+          <t>S048v3_F_TR4_only</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2258</v>
+        <v>455</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -9265,28 +9259,28 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.9019</v>
+        <v>4.0744</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5548999999999999</v>
+        <v>1.4673</v>
       </c>
       <c r="F13" t="n">
-        <v>1.466</v>
+        <v>11.3139</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.6770</t>
+          <t>0.0070</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S048v3_E_no_Bethesda_VI</t>
+          <t>S048v3_G_had_fna</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2599</v>
+        <v>2258</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -9294,13 +9288,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.4169</v>
+        <v>0.5859</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3415</v>
+        <v>0.4671</v>
       </c>
       <c r="F14" t="n">
-        <v>0.509</v>
+        <v>0.7351</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -9311,11 +9305,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S048v3_E_no_Bethesda_VI</t>
+          <t>S048v3_G_had_fna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2599</v>
+        <v>2258</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -9323,17 +9317,17 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.2705</v>
+        <v>0.9019</v>
       </c>
       <c r="E15" t="n">
-        <v>0.8493000000000001</v>
+        <v>0.5548999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>1.9006</v>
+        <v>1.466</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.2440</t>
+          <t>0.6770</t>
         </is>
       </c>
     </row>

</xml_diff>